<commit_message>
fix(testcase): beautify integration arrows with spacing and adjust column width layout
</commit_message>
<xml_diff>
--- a/TestCase/Nhom_9_Integration_Test.xlsx
+++ b/TestCase/Nhom_9_Integration_Test.xlsx
@@ -598,14 +598,14 @@
   <dimension ref="A1:J75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="7" max="7"/>
-    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="8" max="8"/>
     <col width="17" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
   </cols>
@@ -620,7 +620,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Kiểm thử sự tương tác giữa các module: Auth &amp; RBAC, Lịch hẹn ⟷ Khách hàng ⟷ Thợ Spa, POS ⟷ Tồn kho, REST API</t>
+          <t>Kiểm thử sự tương tác giữa các module: Auth &amp; RBAC, Lịch hẹn  &lt;-&gt;  Khách hàng  &lt;-&gt;  Thợ Spa, POS  &lt;-&gt;  Tồn kho, REST API</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Auth Service ⟷ Router Guard ⟷ Staff Page</t>
+          <t>Auth Service  &lt;-&gt;  Router Guard  &lt;-&gt;  Staff Page</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
@@ -746,7 +746,7 @@
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>Auth Service ⟷ App State ⟷ Dashboard Page</t>
+          <t>Auth Service  &lt;-&gt;  App State  &lt;-&gt;  Dashboard Page</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
@@ -797,7 +797,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Auth Service ⟷ Session Persistence ⟷ Header</t>
+          <t>Auth Service  &lt;-&gt;  Session Persistence  &lt;-&gt;  Header</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -848,7 +848,7 @@
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>Auth Service ⟷ Switch Role Controller</t>
+          <t>Auth Service  &lt;-&gt;  Switch Role Controller</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
@@ -899,7 +899,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Auth Service ⟷ Logout Flow ⟷ Login Redirect</t>
+          <t>Auth Service  &lt;-&gt;  Logout Flow  &lt;-&gt;  Login Redirect</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -950,7 +950,7 @@
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>Auth Guard ⟷ Direct URL Access</t>
+          <t>Auth Guard  &lt;-&gt;  Direct URL Access</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
@@ -1001,7 +1001,7 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Auth Service ⟷ Customer Role Rejection</t>
+          <t>Auth Service  &lt;-&gt;  Customer Role Rejection</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -1052,7 +1052,7 @@
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>Auth Service ⟷ Staff Permissions ⟷ PosOrders</t>
+          <t>Auth Service  &lt;-&gt;  Staff Permissions  &lt;-&gt;  PosOrders</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
@@ -1103,7 +1103,7 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Auth Service ⟷ Staff Permissions ⟷ Appointments</t>
+          <t>Auth Service  &lt;-&gt;  Staff Permissions  &lt;-&gt;  Appointments</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
@@ -1154,7 +1154,7 @@
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>Auth Service ⟷ Staff Permissions ⟷ Promotions</t>
+          <t>Auth Service  &lt;-&gt;  Staff Permissions  &lt;-&gt;  Promotions</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
@@ -1205,7 +1205,7 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Appointments Page ⟷ Customer Store ⟷ Pet Store</t>
+          <t>Appointments Page  &lt;-&gt;  Customer Store  &lt;-&gt;  Pet Store</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
@@ -1257,7 +1257,7 @@
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>Appointments Page ⟷ Staff Model ⟷ Calendar View</t>
+          <t>Appointments Page  &lt;-&gt;  Staff Model  &lt;-&gt;  Calendar View</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
@@ -1309,7 +1309,7 @@
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Appointments ⟷ Services Store ⟷ Step 7 Pricing</t>
+          <t>Appointments  &lt;-&gt;  Services Store  &lt;-&gt;  Step 7 Pricing</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
@@ -1360,7 +1360,7 @@
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>Appointments ⟷ Pets Filter by Owner</t>
+          <t>Appointments  &lt;-&gt;  Pets Filter by Owner</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
@@ -1411,7 +1411,7 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Appointments ⟷ Status Transition ⟷ Badge UI</t>
+          <t>Appointments  &lt;-&gt;  Status Transition  &lt;-&gt;  Badge UI</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
@@ -1462,7 +1462,7 @@
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>Appointments ⟷ Status 'Hoàn thành' ⟷ POS Invoicing</t>
+          <t>Appointments  &lt;-&gt;  Status 'Hoàn thành'  &lt;-&gt;  POS Invoicing</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
@@ -1513,7 +1513,7 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Appointments ⟷ Day / Week / Month View Switcher</t>
+          <t>Appointments  &lt;-&gt;  Day / Week / Month View Switcher</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
@@ -1565,7 +1565,7 @@
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>Appointments ⟷ Staff Shift Filter</t>
+          <t>Appointments  &lt;-&gt;  Staff Shift Filter</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
@@ -1616,7 +1616,7 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Appointments ⟷ Status Filter Dropdown</t>
+          <t>Appointments  &lt;-&gt;  Status Filter Dropdown</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
@@ -1667,7 +1667,7 @@
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>Appointments ⟷ Search by Customer Name / Pet</t>
+          <t>Appointments  &lt;-&gt;  Search by Customer Name / Pet</t>
         </is>
       </c>
       <c r="D25" s="12" t="inlineStr">
@@ -1718,7 +1718,7 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Appointments ⟷ Delete Appointment ⟷ State Sync</t>
+          <t>Appointments  &lt;-&gt;  Delete Appointment  &lt;-&gt;  State Sync</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
@@ -1769,7 +1769,7 @@
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>Appointments ⟷ Time Slot Validation Guard</t>
+          <t>Appointments  &lt;-&gt;  Time Slot Validation Guard</t>
         </is>
       </c>
       <c r="D27" s="12" t="inlineStr">
@@ -1820,7 +1820,7 @@
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Appointments ⟷ Multi-step Form Progress Bar</t>
+          <t>Appointments  &lt;-&gt;  Multi-step Form Progress Bar</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
@@ -1871,7 +1871,7 @@
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>Appointments ⟷ Pet Grooming History Sync</t>
+          <t>Appointments  &lt;-&gt;  Pet Grooming History Sync</t>
         </is>
       </c>
       <c r="D29" s="12" t="inlineStr">
@@ -1922,7 +1922,7 @@
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Appointments ⟷ Staff Revenue Stats</t>
+          <t>Appointments  &lt;-&gt;  Staff Revenue Stats</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
@@ -1973,7 +1973,7 @@
       </c>
       <c r="C31" s="12" t="inlineStr">
         <is>
-          <t>Appointments ⟷ Global Search Synchronization</t>
+          <t>Appointments  &lt;-&gt;  Global Search Synchronization</t>
         </is>
       </c>
       <c r="D31" s="12" t="inlineStr">
@@ -2024,7 +2024,7 @@
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>POS Orders ⟷ Products Store (Inventory)</t>
+          <t>POS Orders  &lt;-&gt;  Products Store (Inventory)</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
@@ -2076,7 +2076,7 @@
       </c>
       <c r="C33" s="12" t="inlineStr">
         <is>
-          <t>POS Orders ⟷ Inventory Out-of-Stock Guard</t>
+          <t>POS Orders  &lt;-&gt;  Inventory Out-of-Stock Guard</t>
         </is>
       </c>
       <c r="D33" s="12" t="inlineStr">
@@ -2127,7 +2127,7 @@
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>POS Orders ⟷ Customer Search Autocomplete</t>
+          <t>POS Orders  &lt;-&gt;  Customer Search Autocomplete</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
@@ -2178,7 +2178,7 @@
       </c>
       <c r="C35" s="12" t="inlineStr">
         <is>
-          <t>POS Orders ⟷ Quick Customer Creation</t>
+          <t>POS Orders  &lt;-&gt;  Quick Customer Creation</t>
         </is>
       </c>
       <c r="D35" s="12" t="inlineStr">
@@ -2229,7 +2229,7 @@
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>POS Orders ⟷ Product / Service Tab Switcher</t>
+          <t>POS Orders  &lt;-&gt;  Product / Service Tab Switcher</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
@@ -2280,7 +2280,7 @@
       </c>
       <c r="C37" s="12" t="inlineStr">
         <is>
-          <t>POS Orders ⟷ Category Filter Dropdown</t>
+          <t>POS Orders  &lt;-&gt;  Category Filter Dropdown</t>
         </is>
       </c>
       <c r="D37" s="12" t="inlineStr">
@@ -2331,7 +2331,7 @@
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>POS Orders ⟷ Live Cart Quantity Modifier</t>
+          <t>POS Orders  &lt;-&gt;  Live Cart Quantity Modifier</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
@@ -2382,7 +2382,7 @@
       </c>
       <c r="C39" s="12" t="inlineStr">
         <is>
-          <t>POS Orders ⟷ Remove Cart Item Flow</t>
+          <t>POS Orders  &lt;-&gt;  Remove Cart Item Flow</t>
         </is>
       </c>
       <c r="D39" s="12" t="inlineStr">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>POS Orders ⟷ Clear All Cart Items</t>
+          <t>POS Orders  &lt;-&gt;  Clear All Cart Items</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
@@ -2484,7 +2484,7 @@
       </c>
       <c r="C41" s="12" t="inlineStr">
         <is>
-          <t>POS Orders ⟷ Promotions Store (Voucher)</t>
+          <t>POS Orders  &lt;-&gt;  Promotions Store (Voucher)</t>
         </is>
       </c>
       <c r="D41" s="12" t="inlineStr">
@@ -2536,7 +2536,7 @@
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>POS Orders ⟷ Payment Method Selector</t>
+          <t>POS Orders  &lt;-&gt;  Payment Method Selector</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
@@ -2587,7 +2587,7 @@
       </c>
       <c r="C43" s="12" t="inlineStr">
         <is>
-          <t>POS Orders ⟷ Invoice Drawer Viewer</t>
+          <t>POS Orders  &lt;-&gt;  Invoice Drawer Viewer</t>
         </is>
       </c>
       <c r="D43" s="12" t="inlineStr">
@@ -2638,7 +2638,7 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>POS Orders ⟷ Printable Invoice Integration</t>
+          <t>POS Orders  &lt;-&gt;  Printable Invoice Integration</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
@@ -2689,7 +2689,7 @@
       </c>
       <c r="C45" s="12" t="inlineStr">
         <is>
-          <t>POS Orders ⟷ Order Status Dropdown</t>
+          <t>POS Orders  &lt;-&gt;  Order Status Dropdown</t>
         </is>
       </c>
       <c r="D45" s="12" t="inlineStr">
@@ -2740,7 +2740,7 @@
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>POS Orders ⟷ Search by Code &amp; Customer</t>
+          <t>POS Orders  &lt;-&gt;  Search by Code &amp; Customer</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
@@ -2791,7 +2791,7 @@
       </c>
       <c r="C47" s="12" t="inlineStr">
         <is>
-          <t>POS Orders ⟷ Filter by Status Dropdown</t>
+          <t>POS Orders  &lt;-&gt;  Filter by Status Dropdown</t>
         </is>
       </c>
       <c r="D47" s="12" t="inlineStr">
@@ -2842,7 +2842,7 @@
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>Customers Page ⟷ Pets Page Relationship</t>
+          <t>Customers Page  &lt;-&gt;  Pets Page Relationship</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
@@ -2893,7 +2893,7 @@
       </c>
       <c r="C49" s="12" t="inlineStr">
         <is>
-          <t>Customers Page ⟷ Quick Add Customer Modal</t>
+          <t>Customers Page  &lt;-&gt;  Quick Add Customer Modal</t>
         </is>
       </c>
       <c r="D49" s="12" t="inlineStr">
@@ -2945,7 +2945,7 @@
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>Customers Page ⟷ Tier Badge Color Mapping</t>
+          <t>Customers Page  &lt;-&gt;  Tier Badge Color Mapping</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
@@ -2995,7 +2995,7 @@
       </c>
       <c r="C51" s="12" t="inlineStr">
         <is>
-          <t>Customers Page ⟷ Search by Phone &amp; Code</t>
+          <t>Customers Page  &lt;-&gt;  Search by Phone &amp; Code</t>
         </is>
       </c>
       <c r="D51" s="12" t="inlineStr">
@@ -3046,7 +3046,7 @@
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>Pets Page ⟷ Grid / Table View Switcher</t>
+          <t>Pets Page  &lt;-&gt;  Grid / Table View Switcher</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
@@ -3097,7 +3097,7 @@
       </c>
       <c r="C53" s="12" t="inlineStr">
         <is>
-          <t>Pets Page ⟷ Add Pet Modal</t>
+          <t>Pets Page  &lt;-&gt;  Add Pet Modal</t>
         </is>
       </c>
       <c r="D53" s="12" t="inlineStr">
@@ -3149,7 +3149,7 @@
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>Pets Page ⟷ Species Icon Display</t>
+          <t>Pets Page  &lt;-&gt;  Species Icon Display</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
@@ -3199,7 +3199,7 @@
       </c>
       <c r="C55" s="12" t="inlineStr">
         <is>
-          <t>Customers Page ⟷ Delete Customer Cascade</t>
+          <t>Customers Page  &lt;-&gt;  Delete Customer Cascade</t>
         </is>
       </c>
       <c r="D55" s="12" t="inlineStr">
@@ -3250,7 +3250,7 @@
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>CRM Module ⟷ Appointment History Scan</t>
+          <t>CRM Module  &lt;-&gt;  Appointment History Scan</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
@@ -3301,7 +3301,7 @@
       </c>
       <c r="C57" s="12" t="inlineStr">
         <is>
-          <t>CRM Module ⟷ Send Reminder Action</t>
+          <t>CRM Module  &lt;-&gt;  Send Reminder Action</t>
         </is>
       </c>
       <c r="D57" s="12" t="inlineStr">
@@ -3352,7 +3352,7 @@
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>Promotions Page ⟷ Create Voucher Modal</t>
+          <t>Promotions Page  &lt;-&gt;  Create Voucher Modal</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
@@ -3404,7 +3404,7 @@
       </c>
       <c r="C59" s="12" t="inlineStr">
         <is>
-          <t>Promotions Page ⟷ Copy Code to Clipboard</t>
+          <t>Promotions Page  &lt;-&gt;  Copy Code to Clipboard</t>
         </is>
       </c>
       <c r="D59" s="12" t="inlineStr">
@@ -3455,7 +3455,7 @@
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>Promotions ⟷ POS Voucher Validation</t>
+          <t>Promotions  &lt;-&gt;  POS Voucher Validation</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
@@ -3506,7 +3506,7 @@
       </c>
       <c r="C61" s="12" t="inlineStr">
         <is>
-          <t>Notifications ⟷ StoreContext Badge</t>
+          <t>Notifications  &lt;-&gt;  StoreContext Badge</t>
         </is>
       </c>
       <c r="D61" s="12" t="inlineStr">
@@ -3557,7 +3557,7 @@
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>Frontend ⟷ Backend API GET /api/products</t>
+          <t>Frontend  &lt;-&gt;  Backend API GET /api/products</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="C63" s="12" t="inlineStr">
         <is>
-          <t>Frontend ⟷ Backend API GET /api/services</t>
+          <t>Frontend  &lt;-&gt;  Backend API GET /api/services</t>
         </is>
       </c>
       <c r="D63" s="12" t="inlineStr">
@@ -3658,7 +3658,7 @@
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>Frontend ⟷ Backend API GET /api/customers</t>
+          <t>Frontend  &lt;-&gt;  Backend API GET /api/customers</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
@@ -3708,7 +3708,7 @@
       </c>
       <c r="C65" s="12" t="inlineStr">
         <is>
-          <t>Frontend ⟷ Backend API GET /api/pets</t>
+          <t>Frontend  &lt;-&gt;  Backend API GET /api/pets</t>
         </is>
       </c>
       <c r="D65" s="12" t="inlineStr">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>Frontend ⟷ Backend API GET /api/appointments</t>
+          <t>Frontend  &lt;-&gt;  Backend API GET /api/appointments</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
@@ -3808,7 +3808,7 @@
       </c>
       <c r="C67" s="12" t="inlineStr">
         <is>
-          <t>Frontend ⟷ Backend API POST /api/orders</t>
+          <t>Frontend  &lt;-&gt;  Backend API POST /api/orders</t>
         </is>
       </c>
       <c r="D67" s="12" t="inlineStr">
@@ -3858,7 +3858,7 @@
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>Frontend ⟷ Backend API GET /api/dashboard/stats</t>
+          <t>Frontend  &lt;-&gt;  Backend API GET /api/dashboard/stats</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C69" s="12" t="inlineStr">
         <is>
-          <t>Backend Express ⟷ Swagger UI Documentation</t>
+          <t>Backend Express  &lt;-&gt;  Swagger UI Documentation</t>
         </is>
       </c>
       <c r="D69" s="12" t="inlineStr">
@@ -3958,7 +3958,7 @@
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>Dashboard KPI ⟷ Orders Store ⟷ Revenue Chart</t>
+          <t>Dashboard KPI  &lt;-&gt;  Orders Store  &lt;-&gt;  Revenue Chart</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
@@ -4009,7 +4009,7 @@
       </c>
       <c r="C71" s="12" t="inlineStr">
         <is>
-          <t>Dashboard ⟷ Appointments Store ⟷ Today Schedule Widget</t>
+          <t>Dashboard  &lt;-&gt;  Appointments Store  &lt;-&gt;  Today Schedule Widget</t>
         </is>
       </c>
       <c r="D71" s="12" t="inlineStr">
@@ -4060,7 +4060,7 @@
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>Sidebar Navigation ⟷ Router Guard ⟷ Page View</t>
+          <t>Sidebar Navigation  &lt;-&gt;  Router Guard  &lt;-&gt;  Page View</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
@@ -4111,7 +4111,7 @@
       </c>
       <c r="C73" s="12" t="inlineStr">
         <is>
-          <t>Header Quick Search ⟷ Global State Filter</t>
+          <t>Header Quick Search  &lt;-&gt;  Global State Filter</t>
         </is>
       </c>
       <c r="D73" s="12" t="inlineStr">
@@ -4162,7 +4162,7 @@
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
-          <t>Responsive Layout ⟷ Mobile Drawer ⟷ Overlay</t>
+          <t>Responsive Layout  &lt;-&gt;  Mobile Drawer  &lt;-&gt;  Overlay</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr">
@@ -4213,7 +4213,7 @@
       </c>
       <c r="C75" s="12" t="inlineStr">
         <is>
-          <t>LocalStorage Sync ⟷ Theme/Filter Preference</t>
+          <t>LocalStorage Sync  &lt;-&gt;  Theme/Filter Preference</t>
         </is>
       </c>
       <c r="D75" s="12" t="inlineStr">

</xml_diff>